<commit_message>
🔄 Atualização completa 29/06/2026 17:39
</commit_message>
<xml_diff>
--- a/Imoveis_Grupos.xlsx
+++ b/Imoveis_Grupos.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Imóveis" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Grupos" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Demandas" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Condomínios" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Imóveis" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Dashboard" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Grupos" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Demandas" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Condomínios" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Imóveis'!$A$1:$N$1</definedName>
@@ -552,7 +552,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O1122"/>
+  <dimension ref="A1:O1130"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -56163,6 +56163,441 @@
         </is>
       </c>
       <c r="O1122" s="14" t="inlineStr"/>
+    </row>
+    <row r="1123">
+      <c r="A1123" s="14" t="inlineStr">
+        <is>
+          <t>29/06/2026, 14:30:17</t>
+        </is>
+      </c>
+      <c r="B1123" s="14" t="inlineStr">
+        <is>
+          <t>Corretores de sucesso 👏🇧🇷🎉🍾🙌🏡</t>
+        </is>
+      </c>
+      <c r="C1123" s="14" t="inlineStr">
+        <is>
+          <t>Mirna Ruas</t>
+        </is>
+      </c>
+      <c r="D1123" s="14" t="inlineStr"/>
+      <c r="E1123" s="14" t="inlineStr">
+        <is>
+          <t>Casa</t>
+        </is>
+      </c>
+      <c r="F1123" s="14" t="inlineStr"/>
+      <c r="G1123" s="14" t="n"/>
+      <c r="H1123" s="14" t="n">
+        <v>3</v>
+      </c>
+      <c r="I1123" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="J1123" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="K1123" s="14" t="n"/>
+      <c r="L1123" s="14" t="n"/>
+      <c r="M1123" s="14" t="inlineStr">
+        <is>
+          <t>Casa maravilhosa no jardim Munique
+✅  03 quartos
+✅  01 suíte 
+✅  02 banheiros
+✅  sala grande
+✅  cozinha
+✅  área gourmet 
+✅  churrasqueira 
+✅  piscina
+200 metros de terreno c/ 149 construção 
+Casa nova   
+Valor 750.000 aceita terreno de menor valor
+🛑Oportunidade para morar e investir! Bairro com alto</t>
+        </is>
+      </c>
+      <c r="N1123" s="14" t="inlineStr">
+        <is>
+          <t>Novo</t>
+        </is>
+      </c>
+      <c r="O1123" s="14" t="inlineStr"/>
+    </row>
+    <row r="1124">
+      <c r="A1124" s="14" t="inlineStr">
+        <is>
+          <t>29/06/2026, 14:33:19</t>
+        </is>
+      </c>
+      <c r="B1124" s="14" t="inlineStr">
+        <is>
+          <t>Maringá Apartamentos 🏘️</t>
+        </is>
+      </c>
+      <c r="C1124" s="14" t="inlineStr">
+        <is>
+          <t>Mariza Schmidt</t>
+        </is>
+      </c>
+      <c r="D1124" s="14" t="inlineStr"/>
+      <c r="E1124" s="14" t="inlineStr">
+        <is>
+          <t>Apartamento</t>
+        </is>
+      </c>
+      <c r="F1124" s="14" t="inlineStr">
+        <is>
+          <t>Jardim Acimação</t>
+        </is>
+      </c>
+      <c r="G1124" s="14" t="n"/>
+      <c r="H1124" s="14" t="n">
+        <v>3</v>
+      </c>
+      <c r="I1124" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="J1124" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="K1124" s="14" t="n"/>
+      <c r="L1124" s="14" t="n">
+        <v>550000</v>
+      </c>
+      <c r="M1124" s="14" t="inlineStr">
+        <is>
+          <t>Semi mobiliado, CRECI J10569, condomínio completo com piscina, academia, área infantil, salão de festas, launderia e sacada</t>
+        </is>
+      </c>
+      <c r="N1124" s="14" t="inlineStr">
+        <is>
+          <t>Novo</t>
+        </is>
+      </c>
+      <c r="O1124" s="14" t="inlineStr"/>
+    </row>
+    <row r="1125">
+      <c r="A1125" s="14" t="inlineStr">
+        <is>
+          <t>29/06/2026, 15:27:43</t>
+        </is>
+      </c>
+      <c r="B1125" s="14" t="inlineStr">
+        <is>
+          <t>Corretores de sucesso 👏🇧🇷🎉🍾🙌🏡</t>
+        </is>
+      </c>
+      <c r="C1125" s="14" t="inlineStr">
+        <is>
+          <t>Mirna Ruas</t>
+        </is>
+      </c>
+      <c r="D1125" s="14" t="inlineStr"/>
+      <c r="E1125" s="14" t="inlineStr">
+        <is>
+          <t>Casa</t>
+        </is>
+      </c>
+      <c r="F1125" s="14" t="inlineStr">
+        <is>
+          <t>Parque das Laranjeiras</t>
+        </is>
+      </c>
+      <c r="G1125" s="14" t="n">
+        <v>400</v>
+      </c>
+      <c r="H1125" s="14" t="n"/>
+      <c r="I1125" s="14" t="n"/>
+      <c r="J1125" s="14" t="n"/>
+      <c r="K1125" s="14" t="n"/>
+      <c r="L1125" s="14" t="n">
+        <v>850000</v>
+      </c>
+      <c r="M1125" s="14" t="inlineStr">
+        <is>
+          <t>Área construída 167m². Espaçosa e arejada. Aceita terreno no mesmo bairro.</t>
+        </is>
+      </c>
+      <c r="N1125" s="14" t="inlineStr">
+        <is>
+          <t>Novo</t>
+        </is>
+      </c>
+      <c r="O1125" s="14" t="inlineStr"/>
+    </row>
+    <row r="1126">
+      <c r="A1126" s="14" t="inlineStr">
+        <is>
+          <t>29/06/2026, 16:10:23</t>
+        </is>
+      </c>
+      <c r="B1126" s="14" t="inlineStr">
+        <is>
+          <t>Imoveis Maringá e Região</t>
+        </is>
+      </c>
+      <c r="C1126" s="14" t="inlineStr">
+        <is>
+          <t>Alison Telles</t>
+        </is>
+      </c>
+      <c r="D1126" s="14" t="inlineStr"/>
+      <c r="E1126" s="14" t="inlineStr">
+        <is>
+          <t>Casa</t>
+        </is>
+      </c>
+      <c r="F1126" s="14" t="inlineStr">
+        <is>
+          <t>Jardim Fregadoli</t>
+        </is>
+      </c>
+      <c r="G1126" s="14" t="n">
+        <v>116</v>
+      </c>
+      <c r="H1126" s="14" t="n">
+        <v>3</v>
+      </c>
+      <c r="I1126" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="J1126" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="K1126" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="L1126" s="14" t="n">
+        <v>890000</v>
+      </c>
+      <c r="M1126" s="14" t="inlineStr">
+        <is>
+          <t>Casa à Venda – Jardim Fregadoli | Maringá/PR
+Imóvel moderno com acabamento de alto padrão, próximo à Avenida Gastão Vidigal e com fácil acesso a mercados, farmácias, restaurantes e demais comércios.
+São 116 m² de construção em um terreno de 170 m²,
+Jacuzzi com hidromassagem para 6 pessoas, além d</t>
+        </is>
+      </c>
+      <c r="N1126" s="14" t="inlineStr">
+        <is>
+          <t>Novo</t>
+        </is>
+      </c>
+      <c r="O1126" s="14" t="inlineStr"/>
+    </row>
+    <row r="1127">
+      <c r="A1127" s="14" t="inlineStr">
+        <is>
+          <t>29/06/2026, 16:10:50</t>
+        </is>
+      </c>
+      <c r="B1127" s="14" t="inlineStr">
+        <is>
+          <t>Corretores de sucesso 👏🇧🇷🎉🍾🙌🏡</t>
+        </is>
+      </c>
+      <c r="C1127" s="14" t="inlineStr">
+        <is>
+          <t>Alison Telles</t>
+        </is>
+      </c>
+      <c r="D1127" s="14" t="inlineStr"/>
+      <c r="E1127" s="14" t="inlineStr">
+        <is>
+          <t>Apartamento</t>
+        </is>
+      </c>
+      <c r="F1127" s="14" t="inlineStr">
+        <is>
+          <t>Zona 08</t>
+        </is>
+      </c>
+      <c r="G1127" s="14" t="n">
+        <v>83</v>
+      </c>
+      <c r="H1127" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="I1127" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="J1127" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="K1127" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="L1127" s="14" t="n">
+        <v>950000</v>
+      </c>
+      <c r="M1127" s="14" t="inlineStr">
+        <is>
+          <t>*EDIFÍCIO MISANO RESIDENZA | ZONA 08 – MARINGÁ*
+Apartamento com 83 m² de área privativa, localizado próximo à Unicesumar e ao EuroGarden.
+• 1 suíte + 1 quarto
+• 2 banheiros
+• Sala de estar e jantar integradas
+• Sacada com churrasqueira a carvão
+• Screen Glass e rede de proteção
+• Sol da manhã
+• Ap</t>
+        </is>
+      </c>
+      <c r="N1127" s="14" t="inlineStr">
+        <is>
+          <t>Novo</t>
+        </is>
+      </c>
+      <c r="O1127" s="14" t="inlineStr"/>
+    </row>
+    <row r="1128">
+      <c r="A1128" s="14" t="inlineStr">
+        <is>
+          <t>29/06/2026, 16:37:30</t>
+        </is>
+      </c>
+      <c r="B1128" s="14" t="inlineStr">
+        <is>
+          <t>Imoveis Maringá e Região</t>
+        </is>
+      </c>
+      <c r="C1128" s="14" t="inlineStr">
+        <is>
+          <t>Odair</t>
+        </is>
+      </c>
+      <c r="D1128" s="14" t="inlineStr"/>
+      <c r="E1128" s="14" t="inlineStr">
+        <is>
+          <t>Apartamento</t>
+        </is>
+      </c>
+      <c r="F1128" s="14" t="inlineStr"/>
+      <c r="G1128" s="14" t="n"/>
+      <c r="H1128" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="I1128" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="J1128" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="K1128" s="14" t="n"/>
+      <c r="L1128" s="14" t="n"/>
+      <c r="M1128" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ÓTIMA OPORTUNIDADE BOM JARDIM EM MARINGÁ ÁREA PRIVATIVA DE 138 METROS ÁREA DO LOTE 200 METROS.  *IMÓVEL COM.                *02 Quartos.                 *01suite Closet.             *02 BAnheiro social     *Sala Pe Direito Alto De 5 metros.      *Cozinha Com pia de Mármore De 2.70 mt e IIha.        </t>
+        </is>
+      </c>
+      <c r="N1128" s="14" t="inlineStr">
+        <is>
+          <t>Novo</t>
+        </is>
+      </c>
+      <c r="O1128" s="14" t="inlineStr"/>
+    </row>
+    <row r="1129">
+      <c r="A1129" s="14" t="inlineStr">
+        <is>
+          <t>29/06/2026, 17:16:17</t>
+        </is>
+      </c>
+      <c r="B1129" s="14" t="inlineStr">
+        <is>
+          <t>Corretores de sucesso 👏🇧🇷🎉🍾🙌🏡</t>
+        </is>
+      </c>
+      <c r="C1129" s="14" t="inlineStr">
+        <is>
+          <t>Edson Do Vale</t>
+        </is>
+      </c>
+      <c r="D1129" s="14" t="inlineStr"/>
+      <c r="E1129" s="14" t="inlineStr">
+        <is>
+          <t>Terreno</t>
+        </is>
+      </c>
+      <c r="F1129" s="14" t="inlineStr">
+        <is>
+          <t>Jardim Dias II</t>
+        </is>
+      </c>
+      <c r="G1129" s="14" t="n">
+        <v>413</v>
+      </c>
+      <c r="H1129" s="14" t="n"/>
+      <c r="I1129" s="14" t="n"/>
+      <c r="J1129" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1129" s="14" t="n"/>
+      <c r="L1129" s="14" t="n">
+        <v>350000</v>
+      </c>
+      <c r="M1129" s="14" t="inlineStr">
+        <is>
+          <t>Esquina das ruas Sebastião de Paula e Silva e Pietrobon. Próximo à Av Américo Belay e Av Morangueira. Dimensões aproximadas 20x20m. Estuda troca parcial por carro ou permuta por casa/apartamento até R$400.000</t>
+        </is>
+      </c>
+      <c r="N1129" s="14" t="inlineStr">
+        <is>
+          <t>Novo</t>
+        </is>
+      </c>
+      <c r="O1129" s="14" t="inlineStr"/>
+    </row>
+    <row r="1130">
+      <c r="A1130" s="14" t="inlineStr">
+        <is>
+          <t>29/06/2026, 17:24:02</t>
+        </is>
+      </c>
+      <c r="B1130" s="14" t="inlineStr">
+        <is>
+          <t>Corretores de sucesso 👏🇧🇷🎉🍾🙌🏡</t>
+        </is>
+      </c>
+      <c r="C1130" s="14" t="inlineStr">
+        <is>
+          <t>Edson Do Vale</t>
+        </is>
+      </c>
+      <c r="D1130" s="14" t="inlineStr"/>
+      <c r="E1130" s="14" t="inlineStr">
+        <is>
+          <t>Apartamento</t>
+        </is>
+      </c>
+      <c r="F1130" s="14" t="inlineStr"/>
+      <c r="G1130" s="14" t="n"/>
+      <c r="H1130" s="14" t="n">
+        <v>3</v>
+      </c>
+      <c r="I1130" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="J1130" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="K1130" s="14" t="n">
+        <v>3</v>
+      </c>
+      <c r="L1130" s="14" t="n">
+        <v>822000</v>
+      </c>
+      <c r="M1130" s="14" t="inlineStr">
+        <is>
+          <t>Urban Yticon, 23º andar, 1 moto na garagem, closed, sacada, churrasqueira, sala, cozinha, lazer completo</t>
+        </is>
+      </c>
+      <c r="N1130" s="14" t="inlineStr">
+        <is>
+          <t>Novo</t>
+        </is>
+      </c>
+      <c r="O1130" s="14" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:N1"/>
@@ -56635,7 +57070,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N37"/>
+  <dimension ref="A1:N41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -57576,6 +58011,181 @@
       <c r="L37" s="14" t="n"/>
       <c r="M37" s="14" t="n"/>
       <c r="N37" s="14" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="14" t="inlineStr">
+        <is>
+          <t>29/06/2026, 15:53:39</t>
+        </is>
+      </c>
+      <c r="B38" s="14" t="inlineStr">
+        <is>
+          <t>Maringá Apartamentos 🏘️</t>
+        </is>
+      </c>
+      <c r="C38" s="14" t="inlineStr">
+        <is>
+          <t>João Brenner</t>
+        </is>
+      </c>
+      <c r="D38" s="14" t="inlineStr"/>
+      <c r="E38" s="14" t="inlineStr">
+        <is>
+          <t>Apartamento</t>
+        </is>
+      </c>
+      <c r="F38" s="14" t="inlineStr"/>
+      <c r="G38" s="14" t="n"/>
+      <c r="H38" s="14" t="n"/>
+      <c r="I38" s="14" t="n"/>
+      <c r="J38" s="14" t="n"/>
+      <c r="K38" s="14" t="n"/>
+      <c r="L38" s="14" t="n">
+        <v>800000</v>
+      </c>
+      <c r="M38" s="14" t="inlineStr">
+        <is>
+          <t>Pessoal,
+Alguém com um VISION pra venda, de preferência que pegue outro apartamento de menor valor , na faixa de R$800mil no negócio?
+Chama no privado.</t>
+        </is>
+      </c>
+      <c r="N38" s="14" t="inlineStr">
+        <is>
+          <t>Nova</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="14" t="inlineStr">
+        <is>
+          <t>29/06/2026, 16:18:48</t>
+        </is>
+      </c>
+      <c r="B39" s="14" t="inlineStr">
+        <is>
+          <t>BUSCA DE IMÓVEIS 🏡</t>
+        </is>
+      </c>
+      <c r="C39" s="14" t="inlineStr">
+        <is>
+          <t>Ludmilla Gargantini</t>
+        </is>
+      </c>
+      <c r="D39" s="14" t="inlineStr"/>
+      <c r="E39" s="14" t="inlineStr">
+        <is>
+          <t>Apartamento</t>
+        </is>
+      </c>
+      <c r="F39" s="14" t="inlineStr"/>
+      <c r="G39" s="14" t="n">
+        <v>100</v>
+      </c>
+      <c r="H39" s="14" t="n"/>
+      <c r="I39" s="14" t="n"/>
+      <c r="J39" s="14" t="n"/>
+      <c r="K39" s="14" t="n"/>
+      <c r="L39" s="14" t="n"/>
+      <c r="M39" s="14" t="inlineStr">
+        <is>
+          <t>Pessoal
+Alguém com apartamento com acessibilidade de 100m² ??
+Enviar no PV por favor</t>
+        </is>
+      </c>
+      <c r="N39" s="14" t="inlineStr">
+        <is>
+          <t>Nova</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="14" t="inlineStr">
+        <is>
+          <t>29/06/2026, 16:19:30</t>
+        </is>
+      </c>
+      <c r="B40" s="14" t="inlineStr">
+        <is>
+          <t>Corretores de sucesso 👏🇧🇷🎉🍾🙌🏡</t>
+        </is>
+      </c>
+      <c r="C40" s="14" t="inlineStr">
+        <is>
+          <t>Denilson corretor</t>
+        </is>
+      </c>
+      <c r="D40" s="14" t="inlineStr"/>
+      <c r="E40" s="14" t="inlineStr">
+        <is>
+          <t>Casa</t>
+        </is>
+      </c>
+      <c r="F40" s="14" t="inlineStr"/>
+      <c r="G40" s="14" t="n"/>
+      <c r="H40" s="14" t="n"/>
+      <c r="I40" s="14" t="n"/>
+      <c r="J40" s="14" t="n"/>
+      <c r="K40" s="14" t="n"/>
+      <c r="L40" s="14" t="n">
+        <v>480000</v>
+      </c>
+      <c r="M40" s="14" t="inlineStr">
+        <is>
+          <t>Cliente procura casa na regiao do Dias ate 480 mil Nova  
+Para visitar amanhã de manhã</t>
+        </is>
+      </c>
+      <c r="N40" s="14" t="inlineStr">
+        <is>
+          <t>Nova</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="14" t="inlineStr">
+        <is>
+          <t>29/06/2026, 16:28:22</t>
+        </is>
+      </c>
+      <c r="B41" s="14" t="inlineStr">
+        <is>
+          <t>Maringá Apartamentos 🏘️</t>
+        </is>
+      </c>
+      <c r="C41" s="14" t="inlineStr">
+        <is>
+          <t>Juliana Brenner Corretora de Imovéis</t>
+        </is>
+      </c>
+      <c r="D41" s="14" t="inlineStr"/>
+      <c r="E41" s="14" t="inlineStr">
+        <is>
+          <t>Apartamento</t>
+        </is>
+      </c>
+      <c r="F41" s="14" t="inlineStr"/>
+      <c r="G41" s="14" t="n"/>
+      <c r="H41" s="14" t="n"/>
+      <c r="I41" s="14" t="n"/>
+      <c r="J41" s="14" t="n"/>
+      <c r="K41" s="14" t="n"/>
+      <c r="L41" s="14" t="n">
+        <v>750000</v>
+      </c>
+      <c r="M41" s="14" t="inlineStr">
+        <is>
+          <t>⚠️⚠️⚠️⚠️⚠️⚠️⚠️Procuro apartamento de *até R$ 750.000,00*, localizado nas Zonas 01, 03, 04, 07 ou 08.
+O imóvel *deve ser novo ou já reformado, com móveis planejados*. Pode estar alugado, pois a compra será para investimento.
+O proprietário *deve aceitar como parte do pagamento uma Toyota Hilux, com</t>
+        </is>
+      </c>
+      <c r="N41" s="14" t="inlineStr">
+        <is>
+          <t>Nova</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Corrigir erros gerar_site.py e sincronizar site
</commit_message>
<xml_diff>
--- a/Imoveis_Grupos.xlsx
+++ b/Imoveis_Grupos.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Imóveis" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Dashboard" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Grupos" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Demandas" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Condomínios" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Imóveis" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Grupos" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Demandas" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Condomínios" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Imóveis'!$A$1:$N$1</definedName>
@@ -552,7 +552,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O1130"/>
+  <dimension ref="A1:O1134"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -56598,6 +56598,237 @@
         </is>
       </c>
       <c r="O1130" s="14" t="inlineStr"/>
+    </row>
+    <row r="1131">
+      <c r="A1131" s="14" t="inlineStr">
+        <is>
+          <t>29/06/2026, 14:30:17</t>
+        </is>
+      </c>
+      <c r="B1131" s="14" t="inlineStr">
+        <is>
+          <t>Corretores de sucesso 👏🇧🇷🎉🍾🙌🏡</t>
+        </is>
+      </c>
+      <c r="C1131" s="14" t="inlineStr">
+        <is>
+          <t>Mirna Ruas</t>
+        </is>
+      </c>
+      <c r="D1131" s="14" t="inlineStr"/>
+      <c r="E1131" s="14" t="inlineStr">
+        <is>
+          <t>Casa</t>
+        </is>
+      </c>
+      <c r="F1131" s="14" t="inlineStr"/>
+      <c r="G1131" s="14" t="n"/>
+      <c r="H1131" s="14" t="n">
+        <v>3</v>
+      </c>
+      <c r="I1131" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="J1131" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="K1131" s="14" t="n"/>
+      <c r="L1131" s="14" t="n"/>
+      <c r="M1131" s="14" t="inlineStr">
+        <is>
+          <t>Casa maravilhosa no jardim Munique
+✅  03 quartos
+✅  01 suíte 
+✅  02 banheiros
+✅  sala grande
+✅  cozinha
+✅  área gourmet 
+✅  churrasqueira 
+✅  piscina
+200 metros de terreno c/ 149 construção 
+Casa nova   
+Valor 750.000 aceita terreno de menor valor
+🛑Oportunidade para morar e investir! Bairro com alto</t>
+        </is>
+      </c>
+      <c r="N1131" s="14" t="inlineStr">
+        <is>
+          <t>Novo</t>
+        </is>
+      </c>
+      <c r="O1131" s="14" t="inlineStr"/>
+    </row>
+    <row r="1132">
+      <c r="A1132" s="14" t="inlineStr">
+        <is>
+          <t>29/06/2026, 16:10:23</t>
+        </is>
+      </c>
+      <c r="B1132" s="14" t="inlineStr">
+        <is>
+          <t>Imoveis Maringá e Região</t>
+        </is>
+      </c>
+      <c r="C1132" s="14" t="inlineStr">
+        <is>
+          <t>Alison Telles</t>
+        </is>
+      </c>
+      <c r="D1132" s="14" t="inlineStr"/>
+      <c r="E1132" s="14" t="inlineStr">
+        <is>
+          <t>Casa</t>
+        </is>
+      </c>
+      <c r="F1132" s="14" t="inlineStr">
+        <is>
+          <t>Jardim Fregadoli</t>
+        </is>
+      </c>
+      <c r="G1132" s="14" t="n">
+        <v>116</v>
+      </c>
+      <c r="H1132" s="14" t="n">
+        <v>3</v>
+      </c>
+      <c r="I1132" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="J1132" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="K1132" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="L1132" s="14" t="n">
+        <v>890000</v>
+      </c>
+      <c r="M1132" s="14" t="inlineStr">
+        <is>
+          <t>Casa à Venda – Jardim Fregadoli | Maringá/PR
+Imóvel moderno com acabamento de alto padrão, próximo à Avenida Gastão Vidigal e com fácil acesso a mercados, farmácias, restaurantes e demais comércios.
+São 116 m² de construção em um terreno de 170 m²,
+Jacuzzi com hidromassagem para 6 pessoas, além d</t>
+        </is>
+      </c>
+      <c r="N1132" s="14" t="inlineStr">
+        <is>
+          <t>Novo</t>
+        </is>
+      </c>
+      <c r="O1132" s="14" t="inlineStr"/>
+    </row>
+    <row r="1133">
+      <c r="A1133" s="14" t="inlineStr">
+        <is>
+          <t>29/06/2026, 16:10:50</t>
+        </is>
+      </c>
+      <c r="B1133" s="14" t="inlineStr">
+        <is>
+          <t>Corretores de sucesso 👏🇧🇷🎉🍾🙌🏡</t>
+        </is>
+      </c>
+      <c r="C1133" s="14" t="inlineStr">
+        <is>
+          <t>Alison Telles</t>
+        </is>
+      </c>
+      <c r="D1133" s="14" t="inlineStr"/>
+      <c r="E1133" s="14" t="inlineStr">
+        <is>
+          <t>Apartamento</t>
+        </is>
+      </c>
+      <c r="F1133" s="14" t="inlineStr">
+        <is>
+          <t>Zona 08</t>
+        </is>
+      </c>
+      <c r="G1133" s="14" t="n">
+        <v>83</v>
+      </c>
+      <c r="H1133" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="I1133" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="J1133" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="K1133" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="L1133" s="14" t="n">
+        <v>950000</v>
+      </c>
+      <c r="M1133" s="14" t="inlineStr">
+        <is>
+          <t>*EDIFÍCIO MISANO RESIDENZA | ZONA 08 – MARINGÁ*
+Apartamento com 83 m² de área privativa, localizado próximo à Unicesumar e ao EuroGarden.
+• 1 suíte + 1 quarto
+• 2 banheiros
+• Sala de estar e jantar integradas
+• Sacada com churrasqueira a carvão
+• Screen Glass e rede de proteção
+• Sol da manhã
+• Ap</t>
+        </is>
+      </c>
+      <c r="N1133" s="14" t="inlineStr">
+        <is>
+          <t>Novo</t>
+        </is>
+      </c>
+      <c r="O1133" s="14" t="inlineStr"/>
+    </row>
+    <row r="1134">
+      <c r="A1134" s="14" t="inlineStr">
+        <is>
+          <t>29/06/2026, 16:37:30</t>
+        </is>
+      </c>
+      <c r="B1134" s="14" t="inlineStr">
+        <is>
+          <t>Imoveis Maringá e Região</t>
+        </is>
+      </c>
+      <c r="C1134" s="14" t="inlineStr">
+        <is>
+          <t>Odair</t>
+        </is>
+      </c>
+      <c r="D1134" s="14" t="inlineStr"/>
+      <c r="E1134" s="14" t="inlineStr">
+        <is>
+          <t>Apartamento</t>
+        </is>
+      </c>
+      <c r="F1134" s="14" t="inlineStr"/>
+      <c r="G1134" s="14" t="n"/>
+      <c r="H1134" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="I1134" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="J1134" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="K1134" s="14" t="n"/>
+      <c r="L1134" s="14" t="n"/>
+      <c r="M1134" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ÓTIMA OPORTUNIDADE BOM JARDIM EM MARINGÁ ÁREA PRIVATIVA DE 138 METROS ÁREA DO LOTE 200 METROS.  *IMÓVEL COM.                *02 Quartos.                 *01suite Closet.             *02 BAnheiro social     *Sala Pe Direito Alto De 5 metros.      *Cozinha Com pia de Mármore De 2.70 mt e IIha.        </t>
+        </is>
+      </c>
+      <c r="N1134" s="14" t="inlineStr">
+        <is>
+          <t>Novo</t>
+        </is>
+      </c>
+      <c r="O1134" s="14" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:N1"/>
@@ -57070,7 +57301,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N41"/>
+  <dimension ref="A1:N45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -58182,6 +58413,181 @@
         </is>
       </c>
       <c r="N41" s="14" t="inlineStr">
+        <is>
+          <t>Nova</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="14" t="inlineStr">
+        <is>
+          <t>29/06/2026, 15:53:39</t>
+        </is>
+      </c>
+      <c r="B42" s="14" t="inlineStr">
+        <is>
+          <t>Maringá Apartamentos 🏘️</t>
+        </is>
+      </c>
+      <c r="C42" s="14" t="inlineStr">
+        <is>
+          <t>João Brenner</t>
+        </is>
+      </c>
+      <c r="D42" s="14" t="inlineStr"/>
+      <c r="E42" s="14" t="inlineStr">
+        <is>
+          <t>Apartamento</t>
+        </is>
+      </c>
+      <c r="F42" s="14" t="inlineStr"/>
+      <c r="G42" s="14" t="n"/>
+      <c r="H42" s="14" t="n"/>
+      <c r="I42" s="14" t="n"/>
+      <c r="J42" s="14" t="n"/>
+      <c r="K42" s="14" t="n"/>
+      <c r="L42" s="14" t="n">
+        <v>800000</v>
+      </c>
+      <c r="M42" s="14" t="inlineStr">
+        <is>
+          <t>Pessoal,
+Alguém com um VISION pra venda, de preferência que pegue outro apartamento de menor valor , na faixa de R$800mil no negócio?
+Chama no privado.</t>
+        </is>
+      </c>
+      <c r="N42" s="14" t="inlineStr">
+        <is>
+          <t>Nova</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="14" t="inlineStr">
+        <is>
+          <t>29/06/2026, 16:18:48</t>
+        </is>
+      </c>
+      <c r="B43" s="14" t="inlineStr">
+        <is>
+          <t>BUSCA DE IMÓVEIS 🏡</t>
+        </is>
+      </c>
+      <c r="C43" s="14" t="inlineStr">
+        <is>
+          <t>Ludmilla Gargantini</t>
+        </is>
+      </c>
+      <c r="D43" s="14" t="inlineStr"/>
+      <c r="E43" s="14" t="inlineStr">
+        <is>
+          <t>Apartamento</t>
+        </is>
+      </c>
+      <c r="F43" s="14" t="inlineStr"/>
+      <c r="G43" s="14" t="n">
+        <v>100</v>
+      </c>
+      <c r="H43" s="14" t="n"/>
+      <c r="I43" s="14" t="n"/>
+      <c r="J43" s="14" t="n"/>
+      <c r="K43" s="14" t="n"/>
+      <c r="L43" s="14" t="n"/>
+      <c r="M43" s="14" t="inlineStr">
+        <is>
+          <t>Pessoal
+Alguém com apartamento com acessibilidade de 100m² ??
+Enviar no PV por favor</t>
+        </is>
+      </c>
+      <c r="N43" s="14" t="inlineStr">
+        <is>
+          <t>Nova</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="14" t="inlineStr">
+        <is>
+          <t>29/06/2026, 16:19:30</t>
+        </is>
+      </c>
+      <c r="B44" s="14" t="inlineStr">
+        <is>
+          <t>Corretores de sucesso 👏🇧🇷🎉🍾🙌🏡</t>
+        </is>
+      </c>
+      <c r="C44" s="14" t="inlineStr">
+        <is>
+          <t>Denilson corretor</t>
+        </is>
+      </c>
+      <c r="D44" s="14" t="inlineStr"/>
+      <c r="E44" s="14" t="inlineStr">
+        <is>
+          <t>Casa</t>
+        </is>
+      </c>
+      <c r="F44" s="14" t="inlineStr"/>
+      <c r="G44" s="14" t="n"/>
+      <c r="H44" s="14" t="n"/>
+      <c r="I44" s="14" t="n"/>
+      <c r="J44" s="14" t="n"/>
+      <c r="K44" s="14" t="n"/>
+      <c r="L44" s="14" t="n">
+        <v>480000</v>
+      </c>
+      <c r="M44" s="14" t="inlineStr">
+        <is>
+          <t>Cliente procura casa na regiao do Dias ate 480 mil Nova  
+Para visitar amanhã de manhã</t>
+        </is>
+      </c>
+      <c r="N44" s="14" t="inlineStr">
+        <is>
+          <t>Nova</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="14" t="inlineStr">
+        <is>
+          <t>29/06/2026, 16:28:22</t>
+        </is>
+      </c>
+      <c r="B45" s="14" t="inlineStr">
+        <is>
+          <t>Maringá Apartamentos 🏘️</t>
+        </is>
+      </c>
+      <c r="C45" s="14" t="inlineStr">
+        <is>
+          <t>Juliana Brenner Corretora de Imovéis</t>
+        </is>
+      </c>
+      <c r="D45" s="14" t="inlineStr"/>
+      <c r="E45" s="14" t="inlineStr">
+        <is>
+          <t>Apartamento</t>
+        </is>
+      </c>
+      <c r="F45" s="14" t="inlineStr"/>
+      <c r="G45" s="14" t="n"/>
+      <c r="H45" s="14" t="n"/>
+      <c r="I45" s="14" t="n"/>
+      <c r="J45" s="14" t="n"/>
+      <c r="K45" s="14" t="n"/>
+      <c r="L45" s="14" t="n">
+        <v>750000</v>
+      </c>
+      <c r="M45" s="14" t="inlineStr">
+        <is>
+          <t>⚠️⚠️⚠️⚠️⚠️⚠️⚠️Procuro apartamento de *até R$ 750.000,00*, localizado nas Zonas 01, 03, 04, 07 ou 08.
+O imóvel *deve ser novo ou já reformado, com móveis planejados*. Pode estar alugado, pois a compra será para investimento.
+O proprietário *deve aceitar como parte do pagamento uma Toyota Hilux, com</t>
+        </is>
+      </c>
+      <c r="N45" s="14" t="inlineStr">
         <is>
           <t>Nova</t>
         </is>

</xml_diff>